<commit_message>
Refactor memory calculation functions and enhance SLA validation features
- Updated `calc_model_mem_gb` to include a safe margin parameter for improved memory estimation.
- Modified `calc_kv_per_session_gb` to account for the ratio of KV heads to attention heads.
- Introduced new functions for calculating Time To First Token (TTFT), generation time, and end-to-end latency.
- Enhanced the `run_sizing` function to validate SLA targets for TTFT and e2e latency, providing recommendations if targets are not met.
- Updated frontend components to display SLA validation results and recommendations, improving user feedback on performance metrics.
</commit_message>
<xml_diff>
--- a/app/reportTemplate.xlsx
+++ b/app/reportTemplate.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="149">
   <si>
     <t>Наименование переменной</t>
   </si>
@@ -100,12 +100,6 @@
     <t>Если модель не использует рассуждения — 0. Для reasoning-модели: 20-50% от макс. бюджета (напр. 4096)</t>
   </si>
   <si>
-    <t>Общее число токенов на запрос (T)</t>
-  </si>
-  <si>
-    <t>Рассчитывается: T = SP + Prp + MRT + A</t>
-  </si>
-  <si>
     <t>Число промптов в сессии (N_prp)</t>
   </si>
   <si>
@@ -151,10 +145,10 @@
     <t>байт</t>
   </si>
   <si>
-    <t>Коэффициент накладных расходов (K_overhead)</t>
+    <t>Safe margin, безопасный отступ по памяти (SM)</t>
   </si>
   <si>
-    <t>1.1–1.2. Учитывает буферы, CUDA-графы, workspace и др.</t>
+    <t>Учитывает служебные буферы фреймворка, выравнивание/фрагментацию памяти, CUDA-графы, рабочие области (workspace) и др. накладные расходы размещения на любом инференс-сервисе (vllm, ollama, TensorRT, etc)</t>
   </si>
   <si>
     <t>-</t>
@@ -230,12 +224,6 @@
   </si>
   <si>
     <t>Из спецификации сервера. Например: 8 GPU A100</t>
-  </si>
-  <si>
-    <t>Число экземпляров модели на сервер (N_count_model)</t>
-  </si>
-  <si>
-    <t>Рассчитывается: ⌊GPU_server / GPU_count_model⌋</t>
   </si>
   <si>
     <t>Множитель TP (Z)</t>
@@ -349,7 +337,7 @@
     <t>0.10–0.25. Консервативно: 0.10–0.15</t>
   </si>
   <si>
-    <t>Пропускная способность аналитическая (prefill, токен/с)</t>
+    <t>Пропускная способность аналитическая prefill (Th_pf_analyt)</t>
   </si>
   <si>
     <t>Рассчитывается: (F_count × η_pf × K_batch) / (FPS + 4×L×H×SL)</t>
@@ -358,16 +346,19 @@
     <t>токен/с</t>
   </si>
   <si>
-    <t>Пропускная способность аналитическая (decode, токен/с)</t>
+    <t>Пропускная способность аналитическая decode (Th_dec_analyt)</t>
   </si>
   <si>
     <t>Рассчитывается: (F_count × η_dec × K_batch) / (FPS + 4×L×H×(SL + (T_dec−1)/2))</t>
   </si>
   <si>
-    <t>Пропускная способность эмпирическая (опционально, 0 = не задано)</t>
+    <t>Пропускная способность эмпирическая prefill (Th_pf)</t>
   </si>
   <si>
     <t>Из публичных бенчмарков (input/prefill). Если задано &gt; 0, используется вместо аналитической</t>
+  </si>
+  <si>
+    <t>Пропускная способность эмпирическая decode (Th_dec)</t>
   </si>
   <si>
     <t>Из публичных бенчмарков (output/decode). Если задано &gt; 0, используется вместо аналитической</t>
@@ -385,7 +376,7 @@
     <t>Пропускная способность сервера (Th_server_comp)</t>
   </si>
   <si>
-    <t>Рассчитывается: N_count_model × C_model</t>
+    <t>Рассчитывается: N_count_TP × C_model</t>
   </si>
   <si>
     <t>RPS на одного пользователя (R)</t>
@@ -406,7 +397,52 @@
     <t>Рассчитывается: ⌈(S_sim × R × K_SLA) / Th_server⌉</t>
   </si>
   <si>
-    <t>7. Итоговое количество серверов</t>
+    <t>7. Проверка подобранных конфигураций серверов по TTFT и e2eLatency</t>
+  </si>
+  <si>
+    <t>Время до генерации первого токена на этапе decode (TTFT_analyt)</t>
+  </si>
+  <si>
+    <t>Рассчитывается: (SL/Th_pf) + (1/Th_dec)</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>Время генерации всех токенов на этапе decode (GenerationTime_analyt)</t>
+  </si>
+  <si>
+    <t>Рассчитывается: T_dec/Th_dec</t>
+  </si>
+  <si>
+    <t>End-to-End показатель Latency без учета задержек сети (e2eLatency_analyt)</t>
+  </si>
+  <si>
+    <t>Рассчитывается: TTFT_analyt + GenerationTime_analyt</t>
+  </si>
+  <si>
+    <t>SLA для времени до генерации первого токена на этапе decode (TTFT_SLA)</t>
+  </si>
+  <si>
+    <t>Определяется исходя из требований к SLA</t>
+  </si>
+  <si>
+    <t>SLA для End-to-End показателя Latency без учета задержек сети (e2eLatency_SLA)</t>
+  </si>
+  <si>
+    <t>Выполнили требование по TTFT_SLA</t>
+  </si>
+  <si>
+    <t>Рассчитывается: ДА, если TTFT_SLA &gt;= TTFT_analyt, иначе НЕТ</t>
+  </si>
+  <si>
+    <t>Выполнили требование по e2eLatency_SLA</t>
+  </si>
+  <si>
+    <t>Рассчитывается: ДА, если e2eLatency_SLA &gt;= e2eLatency_analyt, иначе НЕТ</t>
+  </si>
+  <si>
+    <t>8. Итоговое количество серверов</t>
   </si>
   <si>
     <t>Итоговое число серверов (Servers_final)</t>
@@ -506,7 +542,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -529,9 +565,15 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
   </cellXfs>
@@ -751,7 +793,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="69.57"/>
+    <col customWidth="1" min="1" max="1" width="77.86"/>
     <col customWidth="1" min="2" max="2" width="96.86"/>
     <col customWidth="1" min="3" max="3" width="28.86"/>
     <col customWidth="1" min="4" max="4" width="16.0"/>
@@ -1375,14 +1417,13 @@
         <v>30</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="9">
-        <f>D13+D14+D16+D15</f>
-        <v>1600</v>
+        <v>10</v>
+      </c>
+      <c r="D17" s="11">
+        <v>5.0</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -1415,13 +1456,14 @@
         <v>32</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="11">
-        <v>5.0</v>
+        <v>15</v>
+      </c>
+      <c r="D18" s="9">
+        <f>D13+D17*(D14+D16+D15)</f>
+        <v>4000</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -1454,11 +1496,10 @@
         <v>34</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="9">
-        <f>D13+D18*(D14+D16+D15)</f>
-        <v>4000</v>
+        <v>10</v>
+      </c>
+      <c r="D19" s="11">
+        <v>32768.0</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>22</v>
@@ -1494,10 +1535,11 @@
         <v>36</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="11">
-        <v>32768.0</v>
+        <v>15</v>
+      </c>
+      <c r="D20" s="9">
+        <f>MIN(D18,D19)</f>
+        <v>4000</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>22</v>
@@ -1526,22 +1568,11 @@
       <c r="AB20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" s="9">
-        <f>MIN(D19,D20)</f>
-        <v>4000</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
@@ -1566,7 +1597,9 @@
       <c r="AB21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="2"/>
+      <c r="A22" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="B22" s="2"/>
       <c r="C22" s="3"/>
       <c r="D22" s="2"/>
@@ -1595,13 +1628,21 @@
       <c r="AB22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
+      <c r="C23" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="11">
+        <v>32.0</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -1627,19 +1668,19 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="11">
-        <v>32.0</v>
+        <v>2.0</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -1665,20 +1706,20 @@
       <c r="AB24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" s="2" t="s">
+      <c r="A25" s="10" t="s">
         <v>44</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="11">
-        <v>2.0</v>
+      <c r="D25" s="12">
+        <v>5.0</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -1703,21 +1744,21 @@
       <c r="AA25" s="2"/>
       <c r="AB25" s="2"/>
     </row>
-    <row r="26">
+    <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="11">
-        <v>1.1</v>
+        <v>1.0</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -1750,13 +1791,14 @@
         <v>50</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="11">
-        <v>1.0</v>
+        <v>15</v>
+      </c>
+      <c r="D27" s="9">
+        <f>(D23*10^9*D24)/(1024^3)*D26+D25</f>
+        <v>64.60464478</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -1782,22 +1824,11 @@
       <c r="AB27" s="2"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" s="9">
-        <f>(D24*10^9*D25)/(1024^3)*D26*D27</f>
-        <v>65.56510925</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -1822,7 +1853,9 @@
       <c r="AB28" s="2"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2"/>
+      <c r="A29" s="4" t="s">
+        <v>52</v>
+      </c>
       <c r="B29" s="2"/>
       <c r="C29" s="3"/>
       <c r="D29" s="2"/>
@@ -1851,13 +1884,21 @@
       <c r="AB29" s="2"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="C30" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
@@ -1886,16 +1927,16 @@
         <v>55</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D31" s="11">
-        <v>2.0</v>
+        <v>64.0</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -1922,16 +1963,16 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D32" s="11">
-        <v>64.0</v>
+        <v>4096.0</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>18</v>
@@ -1961,19 +2002,19 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D33" s="11">
-        <v>4096.0</v>
+        <v>2.0</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -2000,19 +2041,19 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D34" s="11">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
@@ -2044,14 +2085,13 @@
       <c r="B35" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C35" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" s="11">
-        <v>1.0</v>
+      <c r="C35" s="13"/>
+      <c r="D35" s="9">
+        <f>(D30*D31*D32*D20*D33*D34)/(1024^3)</f>
+        <v>3.90625</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
@@ -2077,20 +2117,11 @@
       <c r="AB35" s="2"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36" s="12"/>
-      <c r="D36" s="9">
-        <f>(D31*D32*D33*D21*D34*D35)/(1024^3)</f>
-        <v>3.90625</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -2115,7 +2146,9 @@
       <c r="AB36" s="2"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="2"/>
+      <c r="A37" s="4" t="s">
+        <v>62</v>
+      </c>
       <c r="B37" s="2"/>
       <c r="C37" s="3"/>
       <c r="D37" s="2"/>
@@ -2144,13 +2177,21 @@
       <c r="AB37" s="2"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="2"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
+      <c r="C38" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="11">
+        <v>80.0</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -2185,10 +2226,10 @@
         <v>10</v>
       </c>
       <c r="D39" s="11">
-        <v>80.0</v>
+        <v>0.9</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
@@ -2221,13 +2262,14 @@
         <v>68</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D40" s="11">
-        <v>0.9</v>
+        <v>15</v>
+      </c>
+      <c r="D40" s="9">
+        <f>_xlfn.CEILING.MATH(D27/(D38*D39))</f>
+        <v>1</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
@@ -2260,11 +2302,10 @@
         <v>70</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D41" s="9">
-        <f>_xlfn.CEILING.MATH(D28/(D39*D40))</f>
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="D41" s="11">
+        <v>8.0</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>18</v>
@@ -2302,11 +2343,11 @@
       <c r="C42" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="11">
-        <v>8.0</v>
+      <c r="D42" s="12">
+        <v>4.0</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
@@ -2342,8 +2383,8 @@
         <v>15</v>
       </c>
       <c r="D43" s="9">
-        <f>_xlfn.FLOOR.MATH(D42/D41)</f>
-        <v>8</v>
+        <f>_xlfn.FLOOR.MATH(D41/(D42*D40))</f>
+        <v>2</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>18</v>
@@ -2379,13 +2420,14 @@
         <v>76</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" s="13">
-        <v>4.0</v>
+        <v>15</v>
+      </c>
+      <c r="D44" s="9">
+        <f>D40*D38*D39-D27</f>
+        <v>7.395355225</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -2421,8 +2463,8 @@
         <v>15</v>
       </c>
       <c r="D45" s="9">
-        <f>_xlfn.FLOOR.MATH(D42/(D44*D41))</f>
-        <v>2</v>
+        <f>_xlfn.FLOOR.MATH(D44/D35)</f>
+        <v>1</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>18</v>
@@ -2461,11 +2503,11 @@
         <v>15</v>
       </c>
       <c r="D46" s="9">
-        <f>D41*D39*D40-D28</f>
-        <v>6.434890747</v>
+        <f>D42*D40*D38*D39-D27</f>
+        <v>223.3953552</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
@@ -2501,8 +2543,8 @@
         <v>15</v>
       </c>
       <c r="D47" s="9">
-        <f>_xlfn.FLOOR.MATH(D46/D36)</f>
-        <v>1</v>
+        <f>_xlfn.FLOOR.MATH(D46/D35)</f>
+        <v>57</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>18</v>
@@ -2538,14 +2580,13 @@
         <v>84</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D48" s="9">
-        <f>D44*D41*D39*D40-D28</f>
-        <v>222.4348907</v>
+        <v>10</v>
+      </c>
+      <c r="D48" s="11">
+        <v>10.0</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
@@ -2581,11 +2622,11 @@
         <v>15</v>
       </c>
       <c r="D49" s="9">
-        <f>_xlfn.FLOOR.MATH(D48/D36)</f>
-        <v>56</v>
+        <f>(D47/D45)*((D45+D48)/(D47+D48))</f>
+        <v>9.358208955</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
@@ -2611,21 +2652,11 @@
       <c r="AB49" s="2"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" s="11">
-        <v>10.0</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
@@ -2650,22 +2681,13 @@
       <c r="AB50" s="2"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D51" s="9">
-        <f>(D49/D47)*((D47+D50)/(D49+D50))</f>
-        <v>9.333333333</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="A51" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B51" s="2"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
@@ -2690,11 +2712,22 @@
       <c r="AB51" s="2"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
+      <c r="A52" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D52" s="9">
+        <f>D43*D47</f>
+        <v>114</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
@@ -2719,13 +2752,22 @@
       <c r="AB52" s="2"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B53" s="2"/>
-      <c r="C53" s="3"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
+      <c r="B53" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D53" s="9">
+        <f>_xlfn.CEILING.MATH(D10/D52)</f>
+        <v>22</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
@@ -2750,22 +2792,11 @@
       <c r="AB53" s="2"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D54" s="9">
-        <f>D45*D49</f>
-        <v>112</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>94</v>
-      </c>
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
@@ -2790,22 +2821,13 @@
       <c r="AB54" s="2"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D55" s="9">
-        <f>_xlfn.CEILING.MATH(D10/D54)</f>
-        <v>23</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A55" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
@@ -2830,11 +2852,22 @@
       <c r="AB55" s="2"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
+      <c r="A56" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D56" s="9">
+        <f>2*D23*10^9</f>
+        <v>64000000000</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
@@ -2859,13 +2892,22 @@
       <c r="AB56" s="2"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B57" s="2"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
+      <c r="B57" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D57" s="9">
+        <f>D15+D16</f>
+        <v>400</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
@@ -2891,20 +2933,19 @@
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D58" s="9">
-        <f>2*D24*10^9</f>
-        <v>64000000000</v>
+        <v>10</v>
+      </c>
+      <c r="D58" s="11">
+        <v>312.0</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
@@ -2931,20 +2972,20 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D59" s="9">
-        <f>D15+D16</f>
-        <v>400</v>
+        <f>D40*D58</f>
+        <v>312</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>22</v>
+        <v>101</v>
       </c>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
@@ -2971,19 +3012,19 @@
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D60" s="11">
-        <v>312.0</v>
+        <v>0.2</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>105</v>
+        <v>46</v>
       </c>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
@@ -3016,14 +3057,13 @@
         <v>107</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D61" s="9">
-        <f>D41*D60</f>
-        <v>312</v>
+        <v>10</v>
+      </c>
+      <c r="D61" s="11">
+        <v>0.15</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>105</v>
+        <v>46</v>
       </c>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
@@ -3049,20 +3089,21 @@
       <c r="AB61" s="2"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="2" t="s">
+      <c r="A62" s="10" t="s">
         <v>108</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D62" s="11">
-        <v>0.2</v>
+        <v>15</v>
+      </c>
+      <c r="D62" s="9">
+        <f>(D59*10^12*D60*D49)/(D56+4*D31*D32*D20)</f>
+        <v>8563.064722</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>48</v>
+        <v>110</v>
       </c>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
@@ -3088,20 +3129,21 @@
       <c r="AB62" s="2"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="2" t="s">
+      <c r="A63" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D63" s="9">
+        <f>(D59*10^12*D61*D49)/(D56+4*D31*D32*(D20+(D57-1)/2))</f>
+        <v>6402.65793</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D63" s="11">
-        <v>0.15</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
@@ -3128,20 +3170,19 @@
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D64" s="9">
-        <f>(D61*10^12*D62*D51)/(D58+4*D32*D33*D21)</f>
-        <v>8540.302721</v>
+        <v>10</v>
+      </c>
+      <c r="D64" s="11">
+        <v>0.0</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
@@ -3174,14 +3215,13 @@
         <v>116</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D65" s="9">
-        <f>(D61*10^12*D63*D51)/(D58+4*D32*D33*(D21+(D59-1)/2))</f>
-        <v>6385.638637</v>
+        <v>10</v>
+      </c>
+      <c r="D65" s="11">
+        <v>0.0</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
@@ -3207,20 +3247,21 @@
       <c r="AB65" s="2"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="10" t="s">
+      <c r="A66" s="2" t="s">
         <v>117</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>118</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D66" s="11">
-        <v>0.0</v>
+        <v>15</v>
+      </c>
+      <c r="D66" s="9">
+        <f>1/(D20/IF(D64&gt;0,D64,D62)+D57/IF(D65&gt;0,D65,D63))</f>
+        <v>1.888229891</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
@@ -3246,20 +3287,21 @@
       <c r="AB66" s="2"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B67" s="2" t="s">
+      <c r="A67" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B67" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D67" s="9">
+        <f>D43*D66</f>
+        <v>3.776459782</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D67" s="11">
-        <v>0.0</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
@@ -3286,20 +3328,19 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D68" s="9">
-        <f>1/(D21/IF(D66&gt;0,D66,D64)+D59/IF(D67&gt;0,D67,D65))</f>
-        <v>1.883210673</v>
+        <v>10</v>
+      </c>
+      <c r="D68" s="11">
+        <v>0.02</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
@@ -3326,20 +3367,19 @@
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D69" s="9">
-        <f>D43*D68</f>
-        <v>15.06568538</v>
+        <v>10</v>
+      </c>
+      <c r="D69" s="11">
+        <v>1.25</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>122</v>
+        <v>46</v>
       </c>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
@@ -3366,19 +3406,20 @@
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D70" s="11">
-        <v>0.02</v>
+        <v>15</v>
+      </c>
+      <c r="D70" s="9">
+        <f>_xlfn.CEILING.MATH((D10*D68*D69)/D67)</f>
+        <v>17</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>122</v>
+        <v>18</v>
       </c>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
@@ -3404,21 +3445,11 @@
       <c r="AB70" s="2"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D71" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
@@ -3443,22 +3474,13 @@
       <c r="AB71" s="2"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D72" s="9">
-        <f>_xlfn.CEILING.MATH((D10*D70*D71)/D69)</f>
-        <v>5</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A72" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B72" s="2"/>
+      <c r="C72" s="3"/>
+      <c r="D72" s="2"/>
+      <c r="E72" s="2"/>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
@@ -3483,11 +3505,22 @@
       <c r="AB72" s="2"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
+      <c r="A73" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B73" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D73" s="9">
+        <f>D20/IF(D64&gt;0,D64,D62)+1/IF(D65&gt;0,D65,D63)</f>
+        <v>0.4672786617</v>
+      </c>
+      <c r="E73" s="10" t="s">
+        <v>131</v>
+      </c>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
@@ -3512,13 +3545,22 @@
       <c r="AB73" s="2"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="4" t="s">
+      <c r="A74" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B74" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D74" s="9">
+        <f>D57/IF(D65&gt;0,D65,D63)</f>
+        <v>0.06247405443</v>
+      </c>
+      <c r="E74" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="B74" s="2"/>
-      <c r="C74" s="3"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
@@ -3543,21 +3585,21 @@
       <c r="AB74" s="2"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>133</v>
+      <c r="A75" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B75" s="10" t="s">
+        <v>135</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D75" s="14">
-        <f>MAX(D55,D72)</f>
-        <v>23</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>18</v>
+      <c r="D75" s="9">
+        <f>D73+D74</f>
+        <v>0.5297527162</v>
+      </c>
+      <c r="E75" s="10" t="s">
+        <v>131</v>
       </c>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
@@ -3583,12 +3625,21 @@
       <c r="AB75" s="2"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="2"/>
-      <c r="B76" s="3"/>
-      <c r="C76" s="3"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="2"/>
+      <c r="A76" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B76" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D76" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>131</v>
+      </c>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
@@ -3613,14 +3664,21 @@
       <c r="AB76" s="2"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B77" s="12"/>
-      <c r="C77" s="12"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="2"/>
+      <c r="A77" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B77" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D77" s="12">
+        <v>1.0</v>
+      </c>
+      <c r="E77" s="10" t="s">
+        <v>131</v>
+      </c>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
@@ -3645,14 +3703,20 @@
       <c r="AB77" s="2"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B78" s="12"/>
-      <c r="C78" s="12"/>
-      <c r="D78" s="9"/>
+      <c r="A78" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B78" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D78" s="15" t="str">
+        <f>IF(D76&gt;=D73,"ДА","НЕТ")</f>
+        <v>ДА</v>
+      </c>
       <c r="E78" s="2"/>
-      <c r="F78" s="2"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
@@ -3677,14 +3741,20 @@
       <c r="AB78" s="2"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B79" s="12"/>
-      <c r="C79" s="12"/>
-      <c r="D79" s="14"/>
+      <c r="A79" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B79" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D79" s="15" t="str">
+        <f>IF(D77&gt;=D75,"ДА","НЕТ")</f>
+        <v>ДА</v>
+      </c>
       <c r="E79" s="2"/>
-      <c r="F79" s="2"/>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
@@ -3710,11 +3780,10 @@
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="2"/>
-      <c r="B80" s="3"/>
+      <c r="B80" s="2"/>
       <c r="C80" s="3"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
-      <c r="F80" s="2"/>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
@@ -3739,12 +3808,13 @@
       <c r="AB80" s="2"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="2"/>
-      <c r="B81" s="3"/>
+      <c r="A81" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B81" s="2"/>
       <c r="C81" s="3"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
-      <c r="F81" s="2"/>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
@@ -3769,12 +3839,22 @@
       <c r="AB81" s="2"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="2"/>
-      <c r="B82" s="3"/>
-      <c r="C82" s="3"/>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="2"/>
+      <c r="A82" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D82" s="16">
+        <f>MAX(D53,D70)</f>
+        <v>22</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
@@ -3829,10 +3909,12 @@
       <c r="AB83" s="2"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="2"/>
-      <c r="B84" s="3"/>
-      <c r="C84" s="3"/>
-      <c r="D84" s="2"/>
+      <c r="A84" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B84" s="13"/>
+      <c r="C84" s="13"/>
+      <c r="D84" s="11"/>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
@@ -3859,10 +3941,12 @@
       <c r="AB84" s="2"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="2"/>
-      <c r="B85" s="3"/>
-      <c r="C85" s="3"/>
-      <c r="D85" s="2"/>
+      <c r="A85" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B85" s="13"/>
+      <c r="C85" s="13"/>
+      <c r="D85" s="9"/>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
@@ -3889,10 +3973,12 @@
       <c r="AB85" s="2"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="2"/>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="2"/>
+      <c r="A86" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B86" s="13"/>
+      <c r="C86" s="13"/>
+      <c r="D86" s="16"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
@@ -31518,6 +31604,216 @@
       <c r="AA1006" s="2"/>
       <c r="AB1006" s="2"/>
     </row>
+    <row r="1007" ht="15.75" customHeight="1">
+      <c r="A1007" s="2"/>
+      <c r="B1007" s="3"/>
+      <c r="C1007" s="3"/>
+      <c r="D1007" s="2"/>
+      <c r="E1007" s="2"/>
+      <c r="F1007" s="2"/>
+      <c r="G1007" s="2"/>
+      <c r="H1007" s="2"/>
+      <c r="I1007" s="2"/>
+      <c r="J1007" s="2"/>
+      <c r="K1007" s="2"/>
+      <c r="L1007" s="2"/>
+      <c r="M1007" s="2"/>
+      <c r="N1007" s="2"/>
+      <c r="O1007" s="2"/>
+      <c r="P1007" s="2"/>
+      <c r="Q1007" s="2"/>
+      <c r="R1007" s="2"/>
+      <c r="S1007" s="2"/>
+      <c r="T1007" s="2"/>
+      <c r="U1007" s="2"/>
+      <c r="V1007" s="2"/>
+      <c r="W1007" s="2"/>
+      <c r="X1007" s="2"/>
+      <c r="Y1007" s="2"/>
+      <c r="Z1007" s="2"/>
+      <c r="AA1007" s="2"/>
+      <c r="AB1007" s="2"/>
+    </row>
+    <row r="1008" ht="15.75" customHeight="1">
+      <c r="A1008" s="2"/>
+      <c r="B1008" s="3"/>
+      <c r="C1008" s="3"/>
+      <c r="D1008" s="2"/>
+      <c r="E1008" s="2"/>
+      <c r="F1008" s="2"/>
+      <c r="G1008" s="2"/>
+      <c r="H1008" s="2"/>
+      <c r="I1008" s="2"/>
+      <c r="J1008" s="2"/>
+      <c r="K1008" s="2"/>
+      <c r="L1008" s="2"/>
+      <c r="M1008" s="2"/>
+      <c r="N1008" s="2"/>
+      <c r="O1008" s="2"/>
+      <c r="P1008" s="2"/>
+      <c r="Q1008" s="2"/>
+      <c r="R1008" s="2"/>
+      <c r="S1008" s="2"/>
+      <c r="T1008" s="2"/>
+      <c r="U1008" s="2"/>
+      <c r="V1008" s="2"/>
+      <c r="W1008" s="2"/>
+      <c r="X1008" s="2"/>
+      <c r="Y1008" s="2"/>
+      <c r="Z1008" s="2"/>
+      <c r="AA1008" s="2"/>
+      <c r="AB1008" s="2"/>
+    </row>
+    <row r="1009" ht="15.75" customHeight="1">
+      <c r="A1009" s="2"/>
+      <c r="B1009" s="3"/>
+      <c r="C1009" s="3"/>
+      <c r="D1009" s="2"/>
+      <c r="E1009" s="2"/>
+      <c r="F1009" s="2"/>
+      <c r="G1009" s="2"/>
+      <c r="H1009" s="2"/>
+      <c r="I1009" s="2"/>
+      <c r="J1009" s="2"/>
+      <c r="K1009" s="2"/>
+      <c r="L1009" s="2"/>
+      <c r="M1009" s="2"/>
+      <c r="N1009" s="2"/>
+      <c r="O1009" s="2"/>
+      <c r="P1009" s="2"/>
+      <c r="Q1009" s="2"/>
+      <c r="R1009" s="2"/>
+      <c r="S1009" s="2"/>
+      <c r="T1009" s="2"/>
+      <c r="U1009" s="2"/>
+      <c r="V1009" s="2"/>
+      <c r="W1009" s="2"/>
+      <c r="X1009" s="2"/>
+      <c r="Y1009" s="2"/>
+      <c r="Z1009" s="2"/>
+      <c r="AA1009" s="2"/>
+      <c r="AB1009" s="2"/>
+    </row>
+    <row r="1010" ht="15.75" customHeight="1">
+      <c r="A1010" s="2"/>
+      <c r="B1010" s="3"/>
+      <c r="C1010" s="3"/>
+      <c r="D1010" s="2"/>
+      <c r="E1010" s="2"/>
+      <c r="F1010" s="2"/>
+      <c r="G1010" s="2"/>
+      <c r="H1010" s="2"/>
+      <c r="I1010" s="2"/>
+      <c r="J1010" s="2"/>
+      <c r="K1010" s="2"/>
+      <c r="L1010" s="2"/>
+      <c r="M1010" s="2"/>
+      <c r="N1010" s="2"/>
+      <c r="O1010" s="2"/>
+      <c r="P1010" s="2"/>
+      <c r="Q1010" s="2"/>
+      <c r="R1010" s="2"/>
+      <c r="S1010" s="2"/>
+      <c r="T1010" s="2"/>
+      <c r="U1010" s="2"/>
+      <c r="V1010" s="2"/>
+      <c r="W1010" s="2"/>
+      <c r="X1010" s="2"/>
+      <c r="Y1010" s="2"/>
+      <c r="Z1010" s="2"/>
+      <c r="AA1010" s="2"/>
+      <c r="AB1010" s="2"/>
+    </row>
+    <row r="1011" ht="15.75" customHeight="1">
+      <c r="A1011" s="2"/>
+      <c r="B1011" s="3"/>
+      <c r="C1011" s="3"/>
+      <c r="D1011" s="2"/>
+      <c r="E1011" s="2"/>
+      <c r="F1011" s="2"/>
+      <c r="G1011" s="2"/>
+      <c r="H1011" s="2"/>
+      <c r="I1011" s="2"/>
+      <c r="J1011" s="2"/>
+      <c r="K1011" s="2"/>
+      <c r="L1011" s="2"/>
+      <c r="M1011" s="2"/>
+      <c r="N1011" s="2"/>
+      <c r="O1011" s="2"/>
+      <c r="P1011" s="2"/>
+      <c r="Q1011" s="2"/>
+      <c r="R1011" s="2"/>
+      <c r="S1011" s="2"/>
+      <c r="T1011" s="2"/>
+      <c r="U1011" s="2"/>
+      <c r="V1011" s="2"/>
+      <c r="W1011" s="2"/>
+      <c r="X1011" s="2"/>
+      <c r="Y1011" s="2"/>
+      <c r="Z1011" s="2"/>
+      <c r="AA1011" s="2"/>
+      <c r="AB1011" s="2"/>
+    </row>
+    <row r="1012" ht="15.75" customHeight="1">
+      <c r="A1012" s="2"/>
+      <c r="B1012" s="3"/>
+      <c r="C1012" s="3"/>
+      <c r="D1012" s="2"/>
+      <c r="E1012" s="2"/>
+      <c r="F1012" s="2"/>
+      <c r="G1012" s="2"/>
+      <c r="H1012" s="2"/>
+      <c r="I1012" s="2"/>
+      <c r="J1012" s="2"/>
+      <c r="K1012" s="2"/>
+      <c r="L1012" s="2"/>
+      <c r="M1012" s="2"/>
+      <c r="N1012" s="2"/>
+      <c r="O1012" s="2"/>
+      <c r="P1012" s="2"/>
+      <c r="Q1012" s="2"/>
+      <c r="R1012" s="2"/>
+      <c r="S1012" s="2"/>
+      <c r="T1012" s="2"/>
+      <c r="U1012" s="2"/>
+      <c r="V1012" s="2"/>
+      <c r="W1012" s="2"/>
+      <c r="X1012" s="2"/>
+      <c r="Y1012" s="2"/>
+      <c r="Z1012" s="2"/>
+      <c r="AA1012" s="2"/>
+      <c r="AB1012" s="2"/>
+    </row>
+    <row r="1013" ht="15.75" customHeight="1">
+      <c r="A1013" s="2"/>
+      <c r="B1013" s="3"/>
+      <c r="C1013" s="3"/>
+      <c r="D1013" s="2"/>
+      <c r="E1013" s="2"/>
+      <c r="F1013" s="2"/>
+      <c r="G1013" s="2"/>
+      <c r="H1013" s="2"/>
+      <c r="I1013" s="2"/>
+      <c r="J1013" s="2"/>
+      <c r="K1013" s="2"/>
+      <c r="L1013" s="2"/>
+      <c r="M1013" s="2"/>
+      <c r="N1013" s="2"/>
+      <c r="O1013" s="2"/>
+      <c r="P1013" s="2"/>
+      <c r="Q1013" s="2"/>
+      <c r="R1013" s="2"/>
+      <c r="S1013" s="2"/>
+      <c r="T1013" s="2"/>
+      <c r="U1013" s="2"/>
+      <c r="V1013" s="2"/>
+      <c r="W1013" s="2"/>
+      <c r="X1013" s="2"/>
+      <c r="Y1013" s="2"/>
+      <c r="Z1013" s="2"/>
+      <c r="AA1013" s="2"/>
+      <c r="AB1013" s="2"/>
+    </row>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>

</xml_diff>